<commit_message>
Dashboard update Tue 10/06/2026 14:43
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{686F6182-0044-4F3E-A1C5-715C7528C581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5230C1D6-3BE0-4A9D-9971-AA54ABB13C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1305" yWindow="420" windowWidth="55020" windowHeight="30150" xr2:uid="{2FD253EF-87A7-481C-B5A2-22EC28C94836}"/>
+    <workbookView xWindow="1050" yWindow="570" windowWidth="50475" windowHeight="30150" xr2:uid="{758BAC64-6380-4B43-9B61-98F8DC9092C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -314,7 +314,7 @@
     <t>Rentokil North America dba Terminix</t>
   </si>
   <si>
-    <t>Two (2) x 1 year w/ 6 months notice.</t>
+    <t>One (1) x 1 year w/ 6 months notice.</t>
   </si>
   <si>
     <t>8% after 5 days + 1%/mo interest</t>
@@ -1320,7 +1320,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09B2F968-3B2B-4A70-BAD6-C2BFCDE3B162}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BB12F4C-013C-4914-9833-B22D987E89F5}">
   <dimension ref="A1:AT300"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2300,7 +2300,7 @@
         <v>45782</v>
       </c>
       <c r="Y16" s="16">
-        <v>46538</v>
+        <v>46904</v>
       </c>
       <c r="Z16" s="17"/>
       <c r="AA16" s="18"/>
@@ -2325,7 +2325,7 @@
         <v>91</v>
       </c>
       <c r="AJ16" s="18">
-        <v>46356</v>
+        <v>46721</v>
       </c>
       <c r="AK16" s="20"/>
       <c r="AL16" s="20"/>
@@ -21065,7 +21065,7 @@
         <v>45782</v>
       </c>
       <c r="U258" s="42">
-        <v>46538</v>
+        <v>46904</v>
       </c>
       <c r="V258" s="13">
         <v>0</v>
@@ -21140,7 +21140,7 @@
         <v>45782</v>
       </c>
       <c r="U259" s="16">
-        <v>46538</v>
+        <v>46904</v>
       </c>
       <c r="V259" s="13">
         <v>0</v>
@@ -21167,7 +21167,7 @@
         <v>90</v>
       </c>
       <c r="E260" s="45" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F260" s="45">
         <v>3</v>
@@ -21215,7 +21215,7 @@
         <v>45782</v>
       </c>
       <c r="U260" s="46">
-        <v>46538</v>
+        <v>46904</v>
       </c>
       <c r="V260" s="48">
         <v>0</v>
@@ -21290,7 +21290,7 @@
         <v>45782</v>
       </c>
       <c r="U261" s="51">
-        <v>46538</v>
+        <v>46904</v>
       </c>
       <c r="V261" s="53">
         <v>0</v>

</xml_diff>